<commit_message>
BOM: add RP2354A price (GBP 1.00 = 1.27 USD)
Unit price converted at the 1.27 USD/GBP rate used in HISTORY section 7.
bom.csv totals now include U1: 6.77 / 5.70 USD per board at qty 10 / 50
(excluding DNP U3/U8).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hexpansion_bom.xlsx
+++ b/hardware/hexpansion_bom.xlsx
@@ -550,14 +550,16 @@
         </is>
       </c>
       <c r="J5" s="6" t="n"/>
-      <c r="K5" s="7" t="n"/>
+      <c r="K5" s="7" t="n">
+        <v>1.27</v>
+      </c>
       <c r="L5" s="8">
         <f>IF(G5="Y",F5*K5,0)</f>
         <v/>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>RP2350A with 2MB flash stacked in package (on QSPI CS0) - no external flash needed. Copy Raspberry Pi RP2350 hardware design guide minimal design. Firmware: PICO_FLASH_SIZE_BYTES = 2MB</t>
+          <t>RP2350A with 2MB flash stacked in package (on QSPI CS0) - no external flash needed. Copy Raspberry Pi RP2350 hardware design guide minimal design. Firmware: PICO_FLASH_SIZE_BYTES = 2MB. Unit cost: GBP 1.00 converted at 1.27 USD/GBP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
hardware: trim schematic - drop DDC, microSD, 0R TMDS and extra passives
- Drop HDMI DDC/EDID (U5 PCA9306 + 6 passives): output is fixed
  640x480@60, so nothing to read. HPD kept on GPIO2.
- Drop microSD (J5, 2 pull-ups, 1 cap): frees the second side flat.
- Drop the eight 0R TMDS insurance resistors; GPIO12-19 drive the ESD
  arrays and socket directly, as on the bench.
- Decoupling cut to the Raspberry Pi minimal design (7 x 100nF on 3V3,
  pins 44/45 and 53/54 share); no BOOTSEL pull-up (internal), no RUN
  debounce cap, no extra HDMI 5V / SD caps.
- Spare GPIOs now 3, 4, 5, 8-11 (no-connect).
- ERC clean except the intended HEXP_DET warning; netlist re-verified
  pin-for-pin (337 pins).
- BOMs regenerated: 78 JLC placements, about $5.01/board (was 107, $5.63).
- README/HISTORY updated with the trims and the microSD decision.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hexpansion_bom.xlsx
+++ b/hardware/hexpansion_bom.xlsx
@@ -406,7 +406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="15" min="1" max="2"/>
@@ -513,7 +513,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>C1,C2,C3,C4,C5,C6,C7,C8,C9,C10,C11,C12,C19,C20,C27,C28,C30,C32</t>
+          <t>C1,C2,C3,C4,C5,C6,C7,C10,C11,C12,C20,C32</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
@@ -569,7 +569,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>C13,C14,C15,C31</t>
+          <t>C13,C14,C15</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
       </c>
       <c r="M12" s="3" t="n"/>
     </row>
-    <row r="13" ht="23.85" customHeight="1" s="15">
+    <row r="13" ht="15" customHeight="1" s="15">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Core</t>
@@ -969,7 +969,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>R3,R5,R7,R41,R42,R43,R44,R45,R46,R47</t>
+          <t>R3,R7,R41</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="M13" s="3" t="n"/>
     </row>
-    <row r="14" ht="23.85" customHeight="1" s="15">
+    <row r="14" ht="15" customHeight="1" s="15">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Core</t>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>R4,R21,R22,R23,R24,R25,R26,R27,R28</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>R19,R29</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
@@ -2341,26 +2341,26 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>R30,R31,R48,R49,R50</t>
+          <t>U6,U7</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>HDMI TMDS ESD (0.5 pF)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE (4.7k)</t>
+          <t>TPD4E05U06DQAR</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>USON-10_L2.5-W1.0-P0.50-BL</t>
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
@@ -2369,19 +2369,19 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C138714</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="J37" s="6" t="n">
-        <v>3285378</v>
+        <v>94387</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>0.0011</v>
+        <v>0.0819</v>
       </c>
       <c r="L37" s="8">
         <f>IF(G37="Y",F37*K37,0)</f>
@@ -2392,40 +2392,40 @@
     <row r="38" ht="15" customHeight="1" s="15">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>HDMI Type A</t>
+          <t>Hexpansion edge connector</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>R32,R33</t>
+          <t>C29</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>EEPROM decoupling</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>0402WGF2001TCE (2k)</t>
+          <t>CL05B104KO5NNNC (100nF)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>C0402</t>
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>C4109</t>
+          <t>C1525</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2434,41 +2434,45 @@
         </is>
       </c>
       <c r="J38" s="6" t="n">
-        <v>1661561</v>
+        <v>16407331</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>0.0008</v>
+        <v>0.006</v>
       </c>
       <c r="L38" s="8">
         <f>IF(G38="Y",F38*K38,0)</f>
         <v/>
       </c>
-      <c r="M38" s="3" t="n"/>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>DNP with U10</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="15">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>HDMI Type A</t>
+          <t>Hexpansion edge connector</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>HDMI DDC level shifter</t>
+          <t>Hexpansion edge connector (PCB edge)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>PCA9306DCUR</t>
+          <t>Hexpansion-Connector</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>SSOP-8_L2.0-W2.3-P0.50-LS3.1-BR</t>
+          <t>hexpansion-edge-connector</t>
         </is>
       </c>
       <c r="F39" s="4" t="n">
@@ -2476,68 +2480,60 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>C33196</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="n">
-        <v>19803</v>
-      </c>
-      <c r="K39" s="7" t="n">
-        <v>0.3319</v>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="6" t="n"/>
+      <c r="K39" s="7" t="n"/>
       <c r="L39" s="8">
         <f>IF(G39="Y",F39*K39,0)</f>
         <v/>
       </c>
-      <c r="M39" s="3" t="n"/>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>PCB edge fingers, no part</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="15">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>HDMI Type A</t>
+          <t>Hexpansion edge connector</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>U6,U7</t>
+          <t>U10</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>HDMI TMDS ESD (0.5 pF)</t>
+          <t>Hexpansion ID EEPROM (fallback)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>TPD4E05U06DQAR</t>
+          <t>ZD24C64A-SSGMT (ZD24C64A (fallback))</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>USON-10_L2.5-W1.0-P0.50-BL</t>
+          <t>SOP-8_L4.9-W3.9-P1.27-LS6.0-BL</t>
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>C138714</t>
+          <t>C2896793</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -2546,149 +2542,149 @@
         </is>
       </c>
       <c r="J40" s="6" t="n">
-        <v>94387</v>
+        <v>6312</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.0819</v>
+        <v>0.1419</v>
       </c>
       <c r="L40" s="8">
         <f>IF(G40="Y",F40*K40,0)</f>
         <v/>
       </c>
-      <c r="M40" s="3" t="n"/>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>DNP. Fit only if EEPROM emulation fails</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="15">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Hexpansion edge connector</t>
+          <t>LEDs, test pads, mounting</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>C29</t>
+          <t>H1,H2</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>EEPROM decoupling</t>
+          <t>Mounting holes</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC (100nF)</t>
+          <t>MountingHole</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>C0402</t>
+          <t>MountingHole_2.2mm_M2_Pad_Via</t>
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>C1525</t>
-        </is>
-      </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>Basic</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="n">
-        <v>16407331</v>
-      </c>
-      <c r="K41" s="7" t="n">
-        <v>0.006</v>
-      </c>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="6" t="n"/>
+      <c r="J41" s="6" t="n"/>
+      <c r="K41" s="7" t="n"/>
       <c r="L41" s="8">
         <f>IF(G41="Y",F41*K41,0)</f>
         <v/>
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>DNP with U10</t>
+          <t>Bare pads</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="15">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Hexpansion edge connector</t>
+          <t>LEDs, test pads, mounting</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>LED1,LED2</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Hexpansion edge connector (PCB edge)</t>
+          <t>Power + status LEDs</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Hexpansion-Connector</t>
+          <t>KT-0603R (PWR/STATUS)</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>hexpansion-edge-connector</t>
+          <t>LED-SMD_L1.6-W0.8-R-RD</t>
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="6" t="n"/>
-      <c r="J42" s="6" t="n"/>
-      <c r="K42" s="7" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>C2286</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="n">
+        <v>8154450</v>
+      </c>
+      <c r="K42" s="7" t="n">
+        <v>0.0073</v>
+      </c>
       <c r="L42" s="8">
         <f>IF(G42="Y",F42*K42,0)</f>
         <v/>
       </c>
-      <c r="M42" s="3" t="inlineStr">
-        <is>
-          <t>PCB edge fingers, no part</t>
-        </is>
-      </c>
+      <c r="M42" s="3" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="15">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Hexpansion edge connector</t>
+          <t>LEDs, test pads, mounting</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>LED3</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Hexpansion ID EEPROM (fallback)</t>
+          <t>RGB status LED</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ZD24C64A-SSGMT (ZD24C64A (fallback))</t>
+          <t>SK6805MICRO-J</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>SOP-8_L4.9-W3.9-P1.27-LS6.0-BL</t>
+          <t>LED-SMD_4P-L2.7-W2.4_SK6805MICRO-J</t>
         </is>
       </c>
       <c r="F43" s="4" t="n">
@@ -2696,12 +2692,12 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>C2896793</t>
+          <t>C2909056</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -2710,45 +2706,41 @@
         </is>
       </c>
       <c r="J43" s="6" t="n">
-        <v>6312</v>
+        <v>38882</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>0.1419</v>
+        <v>0.08989999999999999</v>
       </c>
       <c r="L43" s="8">
         <f>IF(G43="Y",F43*K43,0)</f>
         <v/>
       </c>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t>DNP. Fit only if EEPROM emulation fails</t>
-        </is>
-      </c>
+      <c r="M43" s="3" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="15">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>microSD</t>
+          <t>LEDs, test pads, mounting</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>R52</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Qwiic</t>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB(LF)(SN) (Qwiic)</t>
+          <t>0402WGF3300TCE (330R)</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>CONN-SMD_4P-P1.00_SM04B-SRSS-TB-LF-SN</t>
+          <t>R0402</t>
         </is>
       </c>
       <c r="F44" s="4" t="n">
@@ -2761,19 +2753,19 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>C160404</t>
+          <t>C25104</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="J44" s="6" t="n">
-        <v>7284</v>
+        <v>732878</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.2262</v>
+        <v>0.0012</v>
       </c>
       <c r="L44" s="8">
         <f>IF(G44="Y",F44*K44,0)</f>
@@ -2784,27 +2776,27 @@
     <row r="45" ht="15" customHeight="1" s="15">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>microSD</t>
+          <t>LEDs, test pads, mounting</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>TP1</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>microSD socket</t>
+          <t>Test pad</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>TF-01A (microSD)</t>
+          <t>+3V3</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>TF-SMD_TF-01A</t>
+          <t>TestPoint_Pad_D1.0mm</t>
         </is>
       </c>
       <c r="F45" s="4" t="n">
@@ -2812,55 +2804,47 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>C91145</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="J45" s="6" t="n">
-        <v>165996</v>
-      </c>
-      <c r="K45" s="7" t="n">
-        <v>0.192</v>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="6" t="n"/>
+      <c r="J45" s="6" t="n"/>
+      <c r="K45" s="7" t="n"/>
       <c r="L45" s="8">
         <f>IF(G45="Y",F45*K45,0)</f>
         <v/>
       </c>
-      <c r="M45" s="3" t="n"/>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>Bare pads</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="15">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>microSD</t>
+          <t>LEDs, test pads, mounting</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>JP1</t>
+          <t>TP2</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Qwiic pull-up solder jumper</t>
+          <t>Test pad</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Qwiic pull-ups</t>
+          <t>V5_HDMI</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>SolderJumper-2_P1.3mm_Bridged_RoundedPad1.0x1.5mm</t>
+          <t>TestPoint_Pad_D1.0mm</t>
         </is>
       </c>
       <c r="F46" s="4" t="n">
@@ -2879,11 +2863,7 @@
         <f>IF(G46="Y",F46*K46,0)</f>
         <v/>
       </c>
-      <c r="M46" s="3" t="inlineStr">
-        <is>
-          <t>Bare copper jumper, cut to remove Qwiic pull-ups</t>
-        </is>
-      </c>
+      <c r="M46" s="3" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="15">
       <c r="A47" s="3" t="inlineStr">
@@ -2893,26 +2873,26 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>H1,H2</t>
+          <t>TP3</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Mounting holes</t>
+          <t>Test pad</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>MountingHole</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>MountingHole_2.2mm_M2_Pad_Via</t>
+          <t>TestPoint_Pad_D1.0mm</t>
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
@@ -2927,40 +2907,36 @@
         <f>IF(G47="Y",F47*K47,0)</f>
         <v/>
       </c>
-      <c r="M47" s="3" t="inlineStr">
-        <is>
-          <t>Bare pads</t>
-        </is>
-      </c>
+      <c r="M47" s="3" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="15">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>LEDs, test pads, mounting</t>
+          <t>Qwiic</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>LED1,LED2</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Power + status LEDs</t>
+          <t>Qwiic</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>KT-0603R (PWR/STATUS)</t>
+          <t>SM04B-SRSS-TB(LF)(SN) (Qwiic)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>LED-SMD_L1.6-W0.8-R-RD</t>
+          <t>CONN-SMD_4P-P1.00_SM04B-SRSS-TB-LF-SN</t>
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
@@ -2969,19 +2945,19 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>C2286</t>
+          <t>C160404</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="J48" s="6" t="n">
-        <v>8154450</v>
+        <v>7284</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>0.0073</v>
+        <v>0.2262</v>
       </c>
       <c r="L48" s="8">
         <f>IF(G48="Y",F48*K48,0)</f>
@@ -2992,27 +2968,27 @@
     <row r="49" ht="15" customHeight="1" s="15">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>LEDs, test pads, mounting</t>
+          <t>Qwiic</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>LED3</t>
+          <t>JP1</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>RGB status LED</t>
+          <t>Qwiic pull-up solder jumper</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>SK6805MICRO-J</t>
+          <t>Qwiic pull-ups</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>LED-SMD_4P-L2.7-W2.4_SK6805MICRO-J</t>
+          <t>SolderJumper-2_P1.3mm_Bridged_RoundedPad1.0x1.5mm</t>
         </is>
       </c>
       <c r="F49" s="4" t="n">
@@ -3020,40 +2996,32 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>C2909056</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="J49" s="6" t="n">
-        <v>38882</v>
-      </c>
-      <c r="K49" s="7" t="n">
-        <v>0.08989999999999999</v>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="6" t="n"/>
+      <c r="K49" s="7" t="n"/>
       <c r="L49" s="8">
         <f>IF(G49="Y",F49*K49,0)</f>
         <v/>
       </c>
-      <c r="M49" s="3" t="n"/>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>Bare copper jumper, cut to remove Qwiic pull-ups</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="15">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>LEDs, test pads, mounting</t>
+          <t>Qwiic</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>R52</t>
+          <t>R48,R49,R50</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3063,7 +3031,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>0402WGF3300TCE (330R)</t>
+          <t>0402WGF4701TCE (4.7k)</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -3072,7 +3040,7 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
@@ -3081,7 +3049,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>C25104</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -3090,10 +3058,10 @@
         </is>
       </c>
       <c r="J50" s="6" t="n">
-        <v>732878</v>
+        <v>3285378</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>0.0012</v>
+        <v>0.0011</v>
       </c>
       <c r="L50" s="8">
         <f>IF(G50="Y",F50*K50,0)</f>
@@ -3101,247 +3069,114 @@
       </c>
       <c r="M50" s="3" t="n"/>
     </row>
-    <row r="51" ht="15" customHeight="1" s="15">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>LEDs, test pads, mounting</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>TP1</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>Test pad</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>+3V3</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>TestPoint_Pad_D1.0mm</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="n"/>
-      <c r="I51" s="6" t="n"/>
-      <c r="J51" s="6" t="n"/>
-      <c r="K51" s="7" t="n"/>
-      <c r="L51" s="8">
-        <f>IF(G51="Y",F51*K51,0)</f>
-        <v/>
-      </c>
-      <c r="M51" s="3" t="inlineStr">
-        <is>
-          <t>Bare pads</t>
-        </is>
-      </c>
-    </row>
+    <row r="51" s="15"/>
     <row r="52" ht="15" customHeight="1" s="15">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>LEDs, test pads, mounting</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>TP2</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>Test pad</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>V5_HDMI</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>TestPoint_Pad_D1.0mm</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="n"/>
-      <c r="I52" s="6" t="n"/>
-      <c r="J52" s="6" t="n"/>
-      <c r="K52" s="7" t="n"/>
-      <c r="L52" s="8">
-        <f>IF(G52="Y",F52*K52,0)</f>
-        <v/>
-      </c>
-      <c r="M52" s="3" t="n"/>
+      <c r="K52" s="9" t="inlineStr">
+        <is>
+          <t>Assembled line items</t>
+        </is>
+      </c>
+      <c r="L52" s="10">
+        <f>COUNTIF(G5:G50,"Y")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="15">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>LEDs, test pads, mounting</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>TP3</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Test pad</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>GND</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>TestPoint_Pad_D1.0mm</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
-      <c r="J53" s="6" t="n"/>
-      <c r="K53" s="7" t="n"/>
-      <c r="L53" s="8">
-        <f>IF(G53="Y",F53*K53,0)</f>
-        <v/>
-      </c>
-      <c r="M53" s="3" t="n"/>
-    </row>
-    <row r="54" s="15"/>
+      <c r="K53" s="9" t="inlineStr">
+        <is>
+          <t>Unique Extended parts (setup fee each)</t>
+        </is>
+      </c>
+      <c r="L53" s="10">
+        <f>COUNTIF(I5:I50,"Extended")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="15" customHeight="1" s="15">
+      <c r="K54" s="9" t="inlineStr">
+        <is>
+          <t>Assembly setup fee (USD)</t>
+        </is>
+      </c>
+      <c r="L54" s="11" t="n">
+        <v>8</v>
+      </c>
+    </row>
     <row r="55" ht="15" customHeight="1" s="15">
       <c r="K55" s="9" t="inlineStr">
         <is>
-          <t>Assembled line items</t>
-        </is>
-      </c>
-      <c r="L55" s="10">
-        <f>COUNTIF(G5:G53,"Y")</f>
-        <v/>
+          <t>Extended fee per part (USD)</t>
+        </is>
+      </c>
+      <c r="L55" s="11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="15">
       <c r="K56" s="9" t="inlineStr">
         <is>
-          <t>Unique Extended parts (setup fee each)</t>
-        </is>
-      </c>
-      <c r="L56" s="10">
-        <f>COUNTIF(I5:I53,"Extended")</f>
+          <t>Extended parts fee (USD)</t>
+        </is>
+      </c>
+      <c r="L56" s="12">
+        <f>L53*L55</f>
         <v/>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="15">
       <c r="K57" s="9" t="inlineStr">
         <is>
-          <t>Assembly setup fee (USD)</t>
-        </is>
-      </c>
-      <c r="L57" s="11" t="n">
-        <v>8</v>
+          <t>Parts cost per board (USD)</t>
+        </is>
+      </c>
+      <c r="L57" s="12">
+        <f>SUM(L5:L50)</f>
+        <v/>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="15">
       <c r="K58" s="9" t="inlineStr">
         <is>
-          <t>Extended fee per part (USD)</t>
-        </is>
-      </c>
-      <c r="L58" s="11" t="n">
-        <v>3</v>
+          <t>Boards in run</t>
+        </is>
+      </c>
+      <c r="L58" s="13" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="15">
       <c r="K59" s="9" t="inlineStr">
         <is>
-          <t>Extended parts fee (USD)</t>
+          <t>Parts cost for run (USD)</t>
         </is>
       </c>
       <c r="L59" s="12">
-        <f>L56*L58</f>
+        <f>L57*L58</f>
         <v/>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="15">
-      <c r="K60" s="9" t="inlineStr">
-        <is>
-          <t>Parts cost per board (USD)</t>
-        </is>
-      </c>
-      <c r="L60" s="12">
-        <f>SUM(L5:L53)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="15" customHeight="1" s="15">
-      <c r="K61" s="9" t="inlineStr">
-        <is>
-          <t>Boards in run</t>
-        </is>
-      </c>
-      <c r="L61" s="13" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="62" ht="15" customHeight="1" s="15">
-      <c r="K62" s="9" t="inlineStr">
-        <is>
-          <t>Parts cost for run (USD)</t>
-        </is>
-      </c>
-      <c r="L62" s="12">
-        <f>L60*L61</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="15" customHeight="1" s="15">
-      <c r="K63" s="14" t="inlineStr">
+      <c r="K60" s="14" t="inlineStr">
         <is>
           <t>Assumptions: setup fee and Extended fee are placeholders I entered (roughly typical JLCPCB figures, not verified) - update from the current JLCPCB pricing page. Board count is 5 as suggested; PCB fabrication and shipping/VAT are not included.</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="15" customHeight="1" s="15"/>
-    <row r="65" ht="15" customHeight="1" s="15"/>
+    <row r="61" ht="15" customHeight="1" s="15"/>
+    <row r="62" ht="15" customHeight="1" s="15"/>
+    <row r="63" s="15"/>
+    <row r="64" s="15"/>
+    <row r="65" s="15"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="K63:M65"/>
+    <mergeCell ref="K60:M62"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="G5:G53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="I5:I53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I5:I50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Basic,Preferred,Extended,Not at LCSC"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
hardware: backfeed-proof badge reset via open-drain buffer
LS_A previously reached RUN through a 0R link, so the RUN pull-up could
leak into an unpowered badge. LS_A now drives RUN through U11, an
SN74LVC1G07 open-drain buffer (C7829) powered from 3V3_BADGE, with C33
decoupling and R4 (10k) pulling LS_A up to 3V3_BADGE so it idles at
"not reset". With the badge off, the buffer's Ioff spec (<=10 uA) blocks
the path and the RP2354A keeps running from USB.

- lib/jlc: add SN74LVC1G07DBVR symbol
- ERC clean except intended HEXP_DET warning; netlist re-verified
  (344 pins); no resistor links +3V3 to any badge-facing net
- BOMs regenerated: 80 placements, about $5.11/board
- README/HISTORY: close the LS_A/RUN open item

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hexpansion_bom.xlsx
+++ b/hardware/hexpansion_bom.xlsx
@@ -406,7 +406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="15" min="1" max="2"/>
@@ -513,7 +513,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>C1,C2,C3,C4,C5,C6,C7,C10,C11,C12,C20,C32</t>
+          <t>C1,C2,C3,C4,C5,C6,C7,C10,C11,C12,C20,C32,C33</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>R3,R7,R41</t>
+          <t>R3,R4,R7,R41</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
@@ -1025,26 +1025,26 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>SW1,SW2</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>BOOTSEL + RESET buttons</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>0402WGF0000TCE (0R)</t>
+          <t>TS-1088-AR02016 (BOOTSEL/RESET)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>SW-SMD_L3.9-W3.0-P4.45</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>C17168</t>
+          <t>C720477</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1062,20 +1062,16 @@
         </is>
       </c>
       <c r="J14" s="6" t="n">
-        <v>3956017</v>
+        <v>877449</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>0.0011</v>
+        <v>0.0557</v>
       </c>
       <c r="L14" s="8">
         <f>IF(G14="Y",F14*K14,0)</f>
         <v/>
       </c>
-      <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t>R4 = LS_A to RUN link (see schematic notes)</t>
-        </is>
-      </c>
+      <c r="M14" s="3" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1085,26 +1081,26 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SW1,SW2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>BOOTSEL + RESET buttons</t>
+          <t>Microcontroller, 2 MB flash in package</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>TS-1088-AR02016 (BOOTSEL/RESET)</t>
+          <t>RP2354A</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>SW-SMD_L3.9-W3.0-P4.45</t>
+          <t>QFN-60_L7.0-W7.0-P0.40-TL-EP3.4</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
@@ -1113,27 +1109,31 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>C720477</t>
+          <t>C41378174</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>877449</v>
+        <v>6193</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>0.0557</v>
+        <v>1.3097</v>
       </c>
       <c r="L15" s="8">
         <f>IF(G15="Y",F15*K15,0)</f>
         <v/>
       </c>
-      <c r="M15" s="3" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="15">
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Unit price from JLC list; you quoted GBP 1.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="23.85" customHeight="1" s="15">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Core</t>
@@ -1141,22 +1141,22 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U9</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Microcontroller, 2 MB flash in package</t>
+          <t>QSPI PSRAM 8 MB (hand-solder)</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>RP2354A</t>
+          <t>APS6404L-3SQR-SN</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>QFN-60_L7.0-W7.0-P0.40-TL-EP3.4</t>
+          <t>SOIC-8_L4.9-W3.9-P1.27-LS6.0-BL</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
@@ -1164,12 +1164,12 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>C41378174</t>
+          <t>C5333729</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -1178,10 +1178,10 @@
         </is>
       </c>
       <c r="J16" s="6" t="n">
-        <v>6193</v>
+        <v>41</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>1.3097</v>
+        <v>4.3423</v>
       </c>
       <c r="L16" s="8">
         <f>IF(G16="Y",F16*K16,0)</f>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>Unit price from JLC list; you quoted GBP 1.00</t>
+          <t>DNP. SOP-8 3.3 V part (the -ZR is USON-8). Buy separately for hand soldering</t>
         </is>
       </c>
     </row>
@@ -1201,22 +1201,22 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>QSPI PSRAM 8 MB (hand-solder)</t>
+          <t>Badge LS_A -&gt; RUN open-drain buffer</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>APS6404L-3SQR-SN</t>
+          <t>SN74LVC1G07DBVR</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>SOIC-8_L4.9-W3.9-P1.27-LS6.0-BL</t>
+          <t>SOT-23-5_L3.0-W1.7-P0.95-LS2.8-BR</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
@@ -1224,12 +1224,12 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>C5333729</t>
+          <t>C7829</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1238,10 +1238,10 @@
         </is>
       </c>
       <c r="J17" s="6" t="n">
-        <v>41</v>
+        <v>46270</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>4.3423</v>
+        <v>0.0915</v>
       </c>
       <c r="L17" s="8">
         <f>IF(G17="Y",F17*K17,0)</f>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>DNP. SOP-8 3.3 V part (the -ZR is USON-8). Buy separately for hand soldering</t>
+          <t>Badge reset buffer, powered from the badge rail (no backfeed)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
hardware: edge connector back to J1 and locked in place, HDMI now J5
- Schematic: hexpansion edge connector is J1 again (same symbol UUID as
  the J1 footprint already on the PCB, so Update PCB keeps its position);
  HDMI Type A socket renumbered J1 -> J5. ERC and netlist re-verified.
- PCB: J1 edge connector footprint locked at x 98.25, y 100 mm, F.Cu, so
  layout work can't move it accidentally. Position confirmed unchanged.
- BOMs regenerated for the new references; HISTORY lists the connector
  numbering.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hexpansion_bom.xlsx
+++ b/hardware/hexpansion_bom.xlsx
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">

</xml_diff>